<commit_message>
Update New Relic market reports - 2026-10-13 06:34:57
</commit_message>
<xml_diff>
--- a/output/glo-it.xlsx
+++ b/output/glo-it.xlsx
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>3643</v>
+        <v>3903</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-18 02:28:27
</commit_message>
<xml_diff>
--- a/output/glo-it.xlsx
+++ b/output/glo-it.xlsx
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>169</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>664</v>
+        <v>594</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1064</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-19 01:24:45
</commit_message>
<xml_diff>
--- a/output/glo-it.xlsx
+++ b/output/glo-it.xlsx
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>275</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-21 01:28:53
</commit_message>
<xml_diff>
--- a/output/glo-it.xlsx
+++ b/output/glo-it.xlsx
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>426</v>
+        <v>299</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>772</v>
+        <v>781</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">

</xml_diff>